<commit_message>
Draft webpage. Ready for review. Next step host on Firebase
</commit_message>
<xml_diff>
--- a/events/events-2026-27.xlsx
+++ b/events/events-2026-27.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="Rc9bbf4c72bc54af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="Rb6a4c5082db844f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -137,18 +137,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events_2026_27" displayName="Events_2026_27" ref="A1:J4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events_2026_27" displayName="Events_2026_27" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="Event type"/>
     <x:tableColumn id="2" name="Title"/>
-    <x:tableColumn id="3" name="Event URL"/>
-    <x:tableColumn id="4" name="Date display"/>
-    <x:tableColumn id="5" name="Start date"/>
-    <x:tableColumn id="6" name="End date"/>
-    <x:tableColumn id="7" name="Location"/>
-    <x:tableColumn id="8" name="Location URL"/>
-    <x:tableColumn id="9" name="Organisers"/>
-    <x:tableColumn id="10" name="Booking URL"/>
+    <x:tableColumn id="3" name="Speaker"/>
+    <x:tableColumn id="4" name="Event URL"/>
+    <x:tableColumn id="5" name="Date display"/>
+    <x:tableColumn id="6" name="Start date"/>
+    <x:tableColumn id="7" name="End date"/>
+    <x:tableColumn id="8" name="Location"/>
+    <x:tableColumn id="9" name="Location URL"/>
+    <x:tableColumn id="10" name="Organisers"/>
+    <x:tableColumn id="11" name="Booking URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </x:table>
@@ -349,16 +350,17 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="66.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="27.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="27.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="17.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="25.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26.670000076293945" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -369,27 +371,30 @@
         <x:v>Title</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
+        <x:v>Speaker</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
         <x:v>Event URL</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>Date display</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>Start date</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>End date</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>Location</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="I1" s="6" t="str">
         <x:v>Location URL</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="J1" s="6" t="str">
         <x:v>Organisers</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="K1" s="6" t="str">
         <x:v>Booking URL</x:v>
       </x:c>
     </x:row>
@@ -401,25 +406,26 @@
         <x:v>CeMMAP PhD Research Day</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str"/>
-      <x:c r="D2" s="7" t="str">
+      <x:c r="D2" s="7" t="str"/>
+      <x:c r="E2" s="7" t="str">
         <x:v>25 September 2026</x:v>
-      </x:c>
-      <x:c r="E2" s="10" t="n">
-        <x:v>46290</x:v>
       </x:c>
       <x:c r="F2" s="10" t="n">
         <x:v>46290</x:v>
       </x:c>
-      <x:c r="G2" s="7" t="str">
+      <x:c r="G2" s="10" t="n">
+        <x:v>46290</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
         <x:v>UCL</x:v>
       </x:c>
-      <x:c r="H2" s="7" t="str">
+      <x:c r="I2" s="7" t="str">
         <x:v>https://www.ucl.ac.uk/maps</x:v>
       </x:c>
-      <x:c r="I2" s="7" t="str">
+      <x:c r="J2" s="7" t="str">
         <x:v>Liyang Sun</x:v>
       </x:c>
-      <x:c r="J2" s="7" t="str"/>
+      <x:c r="K2" s="7" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -429,81 +435,112 @@
         <x:v>THEBES Optimal Taxation Conference</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str"/>
-      <x:c r="D3" s="8" t="str">
+      <x:c r="D3" s="8" t="str"/>
+      <x:c r="E3" s="8" t="str">
         <x:v>December 2026</x:v>
       </x:c>
-      <x:c r="E3" s="11"/>
       <x:c r="F3" s="11"/>
-      <x:c r="G3" s="8" t="str">
+      <x:c r="G3" s="11"/>
+      <x:c r="H3" s="8" t="str">
         <x:v>TBA</x:v>
       </x:c>
-      <x:c r="H3" s="8" t="str"/>
-      <x:c r="I3" s="8" t="str">
+      <x:c r="I3" s="8" t="str"/>
+      <x:c r="J3" s="8" t="str">
         <x:v>TBA</x:v>
       </x:c>
-      <x:c r="J3" s="8" t="str"/>
+      <x:c r="K3" s="8" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="9" t="str">
+      <x:c r="A4" s="8" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="B4" s="9" t="str">
+      <x:c r="B4" s="8" t="str">
         <x:v>IFS Empirical Industrial Organisation Conference</x:v>
       </x:c>
-      <x:c r="C4" s="9" t="str"/>
-      <x:c r="D4" s="9" t="str">
+      <x:c r="C4" s="8" t="str"/>
+      <x:c r="D4" s="8" t="str"/>
+      <x:c r="E4" s="8" t="str">
         <x:v>Spring 2027</x:v>
       </x:c>
-      <x:c r="E4" s="12"/>
-      <x:c r="F4" s="12"/>
-      <x:c r="G4" s="9" t="str">
+      <x:c r="F4" s="11"/>
+      <x:c r="G4" s="11"/>
+      <x:c r="H4" s="8" t="str">
         <x:v>Institute for Fiscal Studies</x:v>
       </x:c>
-      <x:c r="H4" s="9" t="str">
+      <x:c r="I4" s="8" t="str">
         <x:v>https://ifs.org.uk/about/contact</x:v>
       </x:c>
-      <x:c r="I4" s="9" t="str">
+      <x:c r="J4" s="8" t="str">
         <x:v>Joao Granja (UCL); Lars Nesheim (UCL); Jakob Schneebacher (IFS); Alessandro Iaria (Bristol University)</x:v>
       </x:c>
-      <x:c r="J4" s="9" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>This workbook is the manually maintained source for the Events webpage. Yellow cells need information.</x:v>
-      </x:c>
+      <x:c r="K4" s="8" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="9" t="str">
+        <x:v>Centre for Finance Annual Lecture</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>The End of the Pax Dollar Era</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>Kenneth Rogoff (Harvard University)</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str"/>
+      <x:c r="E5" s="9" t="str">
+        <x:v>4 November 2027, 18:00</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>46695</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="n">
+        <x:v>46695</x:v>
+      </x:c>
+      <x:c r="H5" s="9" t="str">
+        <x:v>TBA</x:v>
+      </x:c>
+      <x:c r="I5" s="9" t="str"/>
+      <x:c r="J5" s="9" t="str">
+        <x:v>Centre for Finance</x:v>
+      </x:c>
+      <x:c r="K5" s="9" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="13" t="str">
-        <x:v>Dates</x:v>
+        <x:v>Notes</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>Date display is shown on the webpage. Add exact Start date and End date when available.</x:v>
+        <x:v>This workbook is the manually maintained source for the Events webpage. Yellow cells need information.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="13" t="str">
+        <x:v>Dates</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>Date display is shown on the webpage. Add exact Start date and End date when available.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="13" t="str">
         <x:v>Organisers</x:v>
       </x:c>
-      <x:c r="B8" s="14" t="str">
+      <x:c r="B9" s="14" t="str">
         <x:v>Separate multiple organisers with semicolons.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C4">
+  <x:conditionalFormatting sqref="D2:D5">
     <x:cfRule type="containsBlanks" priority="1"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G2:G4">
+  <x:conditionalFormatting sqref="H2:H5">
     <x:cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="TBA"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J2:J4">
+  <x:conditionalFormatting sqref="K2:K5">
     <x:cfRule type="containsBlanks" priority="3"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ce51b2944f040db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd69f01a833d4c74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update CeMMAP research day event
</commit_message>
<xml_diff>
--- a/events/events-2026-27.xlsx
+++ b/events/events-2026-27.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="R654733ef97ab47d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="Rcac0b26ed5514c3c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -416,7 +416,7 @@
         <x:v>Research day</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>CeMMAP PhD Research Day</x:v>
+        <x:v>4th Annual UCL – CeMMAP Ph.D./PostDoc Econometrics Research Day</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str"/>
       <x:c r="D2" s="7" t="str"/>
@@ -430,7 +430,7 @@
         <x:v>46290</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>UCL</x:v>
+        <x:v>B20 Jevons Room Drayton House</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
         <x:v>https://www.ucl.ac.uk/maps</x:v>
@@ -617,7 +617,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26e374b088924a5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R086cbe9386bc42f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update seminar schedules, events and visitors; add PhD series and staff portraits
</commit_message>
<xml_diff>
--- a/events/events-2026-27.xlsx
+++ b/events/events-2026-27.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="Rcac0b26ed5514c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="R651f9ee459c947de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -511,7 +511,7 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>UCL Bloomsbury Campus</x:v>
+        <x:v>LT1 Cruciform</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str"/>
       <x:c r="J5" s="9" t="str">
@@ -617,7 +617,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R086cbe9386bc42f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0d9d870fde94bc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>